<commit_message>
add more m-score tests, placeholder for helpers
</commit_message>
<xml_diff>
--- a/testing/run/testing_files/m_score_tests.xlsx
+++ b/testing/run/testing_files/m_score_tests.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\dergun\Downloads\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\dergun\Documents\hfqa_tool\testing\run\testing_files\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{72A9ABC1-48E3-402A-8C3E-F2401262022D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D06C5335-D942-4299-82F3-21E2B4F98F07}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="38280" yWindow="-120" windowWidth="38640" windowHeight="21120" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="M_score_test_cases" sheetId="1" r:id="rId1"/>
@@ -51,12 +51,6 @@
     <t>C37</t>
   </si>
   <si>
-    <t>C04</t>
-  </si>
-  <si>
-    <t>C05</t>
-  </si>
-  <si>
     <t>C42</t>
   </si>
   <si>
@@ -196,6 +190,12 @@
   </si>
   <si>
     <t>[no]</t>
+  </si>
+  <si>
+    <t>C4</t>
+  </si>
+  <si>
+    <t>C5</t>
   </si>
 </sst>
 </file>
@@ -564,48 +564,48 @@
         <v>7</v>
       </c>
       <c r="I1" t="s">
+        <v>55</v>
+      </c>
+      <c r="J1" t="s">
+        <v>56</v>
+      </c>
+      <c r="K1" t="s">
         <v>8</v>
       </c>
-      <c r="J1" t="s">
+      <c r="L1" t="s">
         <v>9</v>
       </c>
-      <c r="K1" t="s">
+      <c r="M1" t="s">
         <v>10</v>
       </c>
-      <c r="L1" t="s">
+      <c r="N1" t="s">
         <v>11</v>
       </c>
-      <c r="M1" t="s">
+      <c r="O1" t="s">
         <v>12</v>
-      </c>
-      <c r="N1" t="s">
-        <v>13</v>
-      </c>
-      <c r="O1" t="s">
-        <v>14</v>
       </c>
     </row>
     <row r="2" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
+        <v>13</v>
+      </c>
+      <c r="B2" t="s">
+        <v>14</v>
+      </c>
+      <c r="C2" t="s">
         <v>15</v>
       </c>
-      <c r="B2" t="s">
+      <c r="D2" t="s">
         <v>16</v>
       </c>
-      <c r="C2" t="s">
+      <c r="E2" t="s">
         <v>17</v>
       </c>
-      <c r="D2" t="s">
+      <c r="F2" t="s">
         <v>18</v>
       </c>
-      <c r="E2" t="s">
-        <v>19</v>
-      </c>
-      <c r="F2" t="s">
-        <v>20</v>
-      </c>
       <c r="G2" t="s">
-        <v>20</v>
+        <v>18</v>
       </c>
       <c r="H2">
         <v>10</v>
@@ -617,42 +617,42 @@
         <v>1000</v>
       </c>
       <c r="K2" t="s">
-        <v>21</v>
+        <v>19</v>
       </c>
       <c r="L2" t="s">
-        <v>22</v>
+        <v>20</v>
       </c>
       <c r="M2">
         <v>20</v>
       </c>
       <c r="N2" t="s">
-        <v>23</v>
+        <v>21</v>
       </c>
       <c r="O2" t="s">
-        <v>24</v>
+        <v>22</v>
       </c>
     </row>
     <row r="3" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
+        <v>23</v>
+      </c>
+      <c r="B3" t="s">
+        <v>24</v>
+      </c>
+      <c r="C3" t="s">
         <v>25</v>
       </c>
-      <c r="B3" t="s">
+      <c r="D3" t="s">
         <v>26</v>
       </c>
-      <c r="C3" t="s">
+      <c r="E3" t="s">
+        <v>17</v>
+      </c>
+      <c r="F3" t="s">
         <v>27</v>
       </c>
-      <c r="D3" t="s">
-        <v>28</v>
-      </c>
-      <c r="E3" t="s">
-        <v>19</v>
-      </c>
-      <c r="F3" t="s">
-        <v>29</v>
-      </c>
       <c r="G3" t="s">
-        <v>29</v>
+        <v>27</v>
       </c>
       <c r="H3">
         <v>8</v>
@@ -664,42 +664,42 @@
         <v>800</v>
       </c>
       <c r="K3" t="s">
-        <v>21</v>
+        <v>19</v>
       </c>
       <c r="L3" t="s">
-        <v>30</v>
+        <v>28</v>
       </c>
       <c r="M3">
         <v>10</v>
       </c>
       <c r="N3" t="s">
-        <v>23</v>
+        <v>21</v>
       </c>
       <c r="O3" t="s">
-        <v>24</v>
+        <v>22</v>
       </c>
     </row>
     <row r="4" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
+        <v>29</v>
+      </c>
+      <c r="B4" t="s">
+        <v>30</v>
+      </c>
+      <c r="C4" t="s">
         <v>31</v>
       </c>
-      <c r="B4" t="s">
+      <c r="D4" t="s">
         <v>32</v>
       </c>
-      <c r="C4" t="s">
+      <c r="E4" t="s">
+        <v>17</v>
+      </c>
+      <c r="F4" t="s">
         <v>33</v>
       </c>
-      <c r="D4" t="s">
-        <v>34</v>
-      </c>
-      <c r="E4" t="s">
-        <v>19</v>
-      </c>
-      <c r="F4" t="s">
-        <v>35</v>
-      </c>
       <c r="G4" t="s">
-        <v>35</v>
+        <v>33</v>
       </c>
       <c r="H4">
         <v>2</v>
@@ -711,42 +711,42 @@
         <v>500</v>
       </c>
       <c r="K4" t="s">
-        <v>36</v>
+        <v>34</v>
       </c>
       <c r="L4" t="s">
-        <v>30</v>
+        <v>28</v>
       </c>
       <c r="M4">
         <v>5</v>
       </c>
       <c r="N4" t="s">
-        <v>37</v>
+        <v>35</v>
       </c>
       <c r="O4" t="s">
-        <v>38</v>
+        <v>36</v>
       </c>
     </row>
     <row r="5" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
+        <v>37</v>
+      </c>
+      <c r="B5" t="s">
+        <v>38</v>
+      </c>
+      <c r="C5" t="s">
         <v>39</v>
       </c>
-      <c r="B5" t="s">
+      <c r="D5" t="s">
         <v>40</v>
       </c>
-      <c r="C5" t="s">
+      <c r="E5" t="s">
+        <v>17</v>
+      </c>
+      <c r="F5" t="s">
         <v>41</v>
       </c>
-      <c r="D5" t="s">
-        <v>42</v>
-      </c>
-      <c r="E5" t="s">
-        <v>19</v>
-      </c>
-      <c r="F5" t="s">
-        <v>43</v>
-      </c>
       <c r="G5" t="s">
-        <v>35</v>
+        <v>33</v>
       </c>
       <c r="H5">
         <v>1</v>
@@ -758,74 +758,74 @@
         <v>300</v>
       </c>
       <c r="K5" t="s">
-        <v>36</v>
+        <v>34</v>
       </c>
       <c r="L5" t="s">
-        <v>44</v>
+        <v>42</v>
       </c>
       <c r="M5">
         <v>1</v>
       </c>
       <c r="N5" t="s">
-        <v>45</v>
+        <v>43</v>
       </c>
       <c r="O5" t="s">
-        <v>46</v>
+        <v>44</v>
       </c>
     </row>
     <row r="6" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
+        <v>45</v>
+      </c>
+      <c r="B6" t="s">
+        <v>46</v>
+      </c>
+      <c r="C6" t="s">
         <v>47</v>
       </c>
-      <c r="B6" t="s">
+      <c r="D6" t="s">
         <v>48</v>
       </c>
-      <c r="C6" t="s">
-        <v>49</v>
-      </c>
-      <c r="D6" t="s">
-        <v>50</v>
-      </c>
       <c r="E6" t="s">
-        <v>19</v>
+        <v>17</v>
       </c>
       <c r="F6" t="s">
-        <v>20</v>
+        <v>18</v>
       </c>
       <c r="G6" t="s">
-        <v>20</v>
+        <v>18</v>
       </c>
       <c r="H6">
         <v>6</v>
       </c>
       <c r="K6" t="s">
+        <v>49</v>
+      </c>
+      <c r="L6" t="s">
+        <v>50</v>
+      </c>
+      <c r="N6" t="s">
         <v>51</v>
       </c>
-      <c r="L6" t="s">
-        <v>52</v>
-      </c>
-      <c r="N6" t="s">
-        <v>53</v>
-      </c>
       <c r="O6" t="s">
-        <v>53</v>
+        <v>51</v>
       </c>
     </row>
     <row r="7" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
+        <v>52</v>
+      </c>
+      <c r="B7" t="s">
+        <v>14</v>
+      </c>
+      <c r="C7" t="s">
+        <v>53</v>
+      </c>
+      <c r="D7" t="s">
+        <v>16</v>
+      </c>
+      <c r="E7" t="s">
         <v>54</v>
-      </c>
-      <c r="B7" t="s">
-        <v>16</v>
-      </c>
-      <c r="C7" t="s">
-        <v>55</v>
-      </c>
-      <c r="D7" t="s">
-        <v>18</v>
-      </c>
-      <c r="E7" t="s">
-        <v>56</v>
       </c>
     </row>
   </sheetData>

</xml_diff>